<commit_message>
feat: enhance project summary with new lines and icons
- Added new icons for project lines including processing, feed reserve, and generator.
- Introduced LINE_ICON mapping to include new line icons.
- Updated deck data structure to include project lines with detailed cost breakdowns.
- Modified financing and cost calculation functions to accommodate new project line data.
- Enhanced slides to display additional information about project lines and their contributions to the total cost.
- Updated JSON data to reflect new project structure and costs.
</commit_message>
<xml_diff>
--- a/data/Кегейли.xlsx
+++ b/data/Кегейли.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB82822-2AF6-4519-9AA5-4BF7681CFB83}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBF60FF-88D8-46AA-AB35-07DB5CB0DEBF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,9 @@
     <sheet name="броллер" sheetId="2" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Жами Лойиҳа Кегели'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Жами Лойиҳа Кегели'!$A$1:$H$35</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="102">
   <si>
     <t>№</t>
   </si>
@@ -811,6 +810,9 @@
   </si>
   <si>
     <t>Дастгох</t>
+  </si>
+  <si>
+    <t>Генератор (движон)           22  дона</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1065,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1096,13 +1098,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1218,7 +1214,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1530,10 +1526,13 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1851,7 +1850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8B84C59-7AA9-41EB-88FC-AD7DB4432DD4}">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="1" customWidth="1"/>
@@ -1917,32 +1916,32 @@
       </c>
     </row>
     <row r="6" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27">
+      <c r="A6" s="107">
         <v>1</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="27">
+      <c r="C6" s="107">
         <v>15</v>
       </c>
-      <c r="D6" s="107">
+      <c r="D6" s="108">
         <f>+D7+D8</f>
         <v>11270</v>
       </c>
-      <c r="E6" s="34">
+      <c r="E6" s="109">
         <f>+E7+E8</f>
         <v>4530</v>
       </c>
-      <c r="F6" s="34">
+      <c r="F6" s="109">
         <f t="shared" ref="F6" si="0">+F7+F8</f>
         <v>3225</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="109">
         <f>+G7+G8</f>
         <v>630</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="109">
         <f>+H7+H8</f>
         <v>2885</v>
       </c>
@@ -1995,33 +1994,33 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="11" customFormat="1" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="20">
+    <row r="9" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="107">
         <v>2</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="107" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="27">
+      <c r="C9" s="107">
         <v>3</v>
       </c>
-      <c r="D9" s="107">
+      <c r="D9" s="108">
         <f>+D10+D11</f>
         <v>3900</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="109">
         <f>+E10+E11</f>
         <v>1740</v>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="109">
         <f>+F10+F11</f>
         <v>1260</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="109">
         <f>+G10+G11</f>
         <v>900</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="109">
         <f t="shared" ref="H9" si="1">+H10+H11</f>
         <v>0</v>
       </c>
@@ -2074,32 +2073,32 @@
       </c>
     </row>
     <row r="12" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27">
+      <c r="A12" s="107">
         <v>3</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="107" t="s">
         <v>98</v>
       </c>
-      <c r="C12" s="27">
+      <c r="C12" s="107">
         <v>10</v>
       </c>
-      <c r="D12" s="107">
+      <c r="D12" s="108">
         <f>+D13+D14</f>
         <v>9520</v>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="109">
         <f>+E13+E14</f>
         <v>3292</v>
       </c>
-      <c r="F12" s="34">
+      <c r="F12" s="109">
         <f>+F13+F14</f>
         <v>2628</v>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="109">
         <f>+G13+G14</f>
         <v>3600</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="109">
         <f>+H13+H14</f>
         <v>0</v>
       </c>
@@ -2153,32 +2152,32 @@
       </c>
     </row>
     <row r="15" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27">
+      <c r="A15" s="107">
         <v>4</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="107" t="s">
         <v>99</v>
       </c>
-      <c r="C15" s="27">
+      <c r="C15" s="107">
         <v>31</v>
       </c>
-      <c r="D15" s="107">
+      <c r="D15" s="108">
         <f>+D16+D17</f>
         <v>14270</v>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="109">
         <f>+E16+E17</f>
         <v>8390</v>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="109">
         <f>+F16+F17</f>
         <v>3360</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="109">
         <f>+G16+G17</f>
         <v>1260</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="109">
         <f>+H16+H17</f>
         <v>1260</v>
       </c>
@@ -2230,30 +2229,30 @@
       </c>
     </row>
     <row r="18" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27">
+      <c r="A18" s="107">
         <v>5</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="107" t="s">
         <v>100</v>
       </c>
-      <c r="C18" s="27"/>
-      <c r="D18" s="107">
+      <c r="C18" s="107"/>
+      <c r="D18" s="108">
         <f>+D19+D20</f>
         <v>5657</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="109">
         <f>+E19+E20</f>
         <v>1200</v>
       </c>
-      <c r="F18" s="34">
+      <c r="F18" s="109">
         <f>+F19+F20</f>
         <v>4457</v>
       </c>
-      <c r="G18" s="34">
+      <c r="G18" s="109">
         <f>+G19+G20</f>
         <v>0</v>
       </c>
-      <c r="H18" s="34">
+      <c r="H18" s="109">
         <f>+H19+H20</f>
         <v>0</v>
       </c>
@@ -2304,160 +2303,294 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    <row r="21" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="107">
         <v>6</v>
       </c>
-      <c r="B21" s="108" t="s">
+      <c r="B21" s="107" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="88">
+      <c r="C21" s="107"/>
+      <c r="D21" s="108">
+        <f>+D22+D23</f>
         <v>6000</v>
       </c>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-    </row>
-    <row r="22" spans="1:8" ht="42" x14ac:dyDescent="0.25">
-      <c r="A22" s="61"/>
-      <c r="B22" s="61" t="s">
+      <c r="E21" s="109">
+        <f>+E22+E23</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="109">
+        <f>+F22+F23</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="109">
+        <f>+G22+G23</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="109">
+        <f>+H22+H23</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="49"/>
+      <c r="D22" s="88">
+        <f>+E22+F22+G22+H22</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="13">
+        <v>0</v>
+      </c>
+      <c r="F22" s="13">
+        <v>0</v>
+      </c>
+      <c r="G22" s="13">
+        <v>0</v>
+      </c>
+      <c r="H22" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="49" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="49"/>
+      <c r="D23" s="88">
+        <f>+E23+F23+G23+H23</f>
+        <v>6000</v>
+      </c>
+      <c r="E23" s="13">
+        <v>0</v>
+      </c>
+      <c r="F23" s="13">
+        <v>0</v>
+      </c>
+      <c r="G23" s="13">
+        <v>0</v>
+      </c>
+      <c r="H23" s="13">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="11" customFormat="1" ht="42" x14ac:dyDescent="0.25">
+      <c r="A24" s="107">
+        <v>7</v>
+      </c>
+      <c r="B24" s="107" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="107"/>
+      <c r="D24" s="109">
+        <f>+D25+D26</f>
+        <v>382.2</v>
+      </c>
+      <c r="E24" s="109">
+        <f>+E25+E26</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="109">
+        <f>+F25+F26</f>
+        <v>382.2</v>
+      </c>
+      <c r="G24" s="109">
+        <f>+G25+G26</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="109">
+        <f>+H25+H26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="49"/>
+      <c r="D25" s="88">
+        <f>+E25+F25+G25+H25</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="13">
+        <v>0</v>
+      </c>
+      <c r="F25" s="13">
+        <v>0</v>
+      </c>
+      <c r="G25" s="13">
+        <v>0</v>
+      </c>
+      <c r="H25" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="49" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="49"/>
+      <c r="D26" s="88">
+        <f>+E26+F26+G26+H26</f>
+        <v>382.2</v>
+      </c>
+      <c r="E26" s="13">
+        <v>0</v>
+      </c>
+      <c r="F26" s="13">
+        <v>382.2</v>
+      </c>
+      <c r="G26" s="13">
+        <v>0</v>
+      </c>
+      <c r="H26" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="42" x14ac:dyDescent="0.25">
+      <c r="A27" s="61"/>
+      <c r="B27" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="61"/>
-      <c r="D22" s="84">
-        <f>+D18+D9+D6+D12+D15+D21</f>
-        <v>50617</v>
-      </c>
-      <c r="E22" s="62">
-        <f t="shared" ref="E22:H24" si="2">+E18+E9+E6</f>
-        <v>7470</v>
-      </c>
-      <c r="F22" s="62">
-        <f t="shared" si="2"/>
-        <v>8942</v>
-      </c>
-      <c r="G22" s="62">
-        <f t="shared" si="2"/>
-        <v>1530</v>
-      </c>
-      <c r="H22" s="62">
-        <f t="shared" si="2"/>
-        <v>2885</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="64"/>
-      <c r="B23" s="65" t="s">
+      <c r="C27" s="61"/>
+      <c r="D27" s="84">
+        <f>+D18+D9+D6+D12+D15+D21+D24</f>
+        <v>50999.199999999997</v>
+      </c>
+      <c r="E27" s="62">
+        <f>+E18+E9+E6+E12+E15+E21+E24</f>
+        <v>19152</v>
+      </c>
+      <c r="F27" s="62">
+        <f>+F18+F9+F6+F12+F15+F21+F24</f>
+        <v>15312.2</v>
+      </c>
+      <c r="G27" s="62">
+        <f>+G18+G9+G6+G12+G15+G21+G24</f>
+        <v>6390</v>
+      </c>
+      <c r="H27" s="62">
+        <f>+H18+H9+H6+H12+H15+H21+H24</f>
+        <v>10145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="64"/>
+      <c r="B28" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="C23" s="65"/>
-      <c r="D23" s="85">
-        <f>+D19+D10+D7+D13+D16</f>
+      <c r="C28" s="65"/>
+      <c r="D28" s="85">
+        <f>+D19+D10+D7+D13+D16+D22+D25</f>
         <v>14245</v>
       </c>
-      <c r="E23" s="63">
-        <f t="shared" si="2"/>
-        <v>3740</v>
-      </c>
-      <c r="F23" s="63">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G23" s="63">
-        <f t="shared" si="2"/>
-        <v>630</v>
-      </c>
-      <c r="H23" s="63">
-        <f t="shared" si="2"/>
-        <v>2885</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="64"/>
-      <c r="B24" s="65" t="s">
+      <c r="E28" s="63">
+        <f>+E19+E10+E7+E13+E16</f>
+        <v>7670</v>
+      </c>
+      <c r="F28" s="63">
+        <f>+F19+F10+F7</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="63">
+        <f>+G19+G10+G7+G13+G16</f>
+        <v>2430</v>
+      </c>
+      <c r="H28" s="63">
+        <f>+H19+H10+H7+H13+H16</f>
+        <v>4145</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="64"/>
+      <c r="B29" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="85">
+      <c r="C29" s="85">
         <f>C6+C9+C12+C15</f>
         <v>59</v>
       </c>
-      <c r="D24" s="85">
-        <f>+D20+D11+D8+D14+D17+D21</f>
-        <v>36372</v>
-      </c>
-      <c r="E24" s="63">
-        <f t="shared" si="2"/>
-        <v>3730</v>
-      </c>
-      <c r="F24" s="63">
-        <f t="shared" si="2"/>
-        <v>8942</v>
-      </c>
-      <c r="G24" s="63">
-        <f t="shared" si="2"/>
-        <v>900</v>
-      </c>
-      <c r="H24" s="63">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="86"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" s="70" customFormat="1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A29" s="68"/>
-      <c r="B29" s="68" t="s">
+      <c r="D29" s="85">
+        <f>+D20+D11+D8+D14+D17+D23+D26</f>
+        <v>36754.199999999997</v>
+      </c>
+      <c r="E29" s="63">
+        <f>+E20+E11+E8+E14+E17</f>
+        <v>11482</v>
+      </c>
+      <c r="F29" s="63">
+        <f>+F20+F11+F8+F14+F17+F24</f>
+        <v>15312.2</v>
+      </c>
+      <c r="G29" s="63">
+        <f>+G20+G11+G8+G14+G17</f>
+        <v>3960</v>
+      </c>
+      <c r="H29" s="63">
+        <f>+H20+H11+H8+H14+H179+H23</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="86"/>
+      <c r="E31" s="67"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="71"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" s="70" customFormat="1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A34" s="68"/>
+      <c r="B34" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="68"/>
-      <c r="D29" s="87">
-        <f>+D24</f>
-        <v>36372</v>
-      </c>
-      <c r="E29" s="68"/>
-      <c r="F29" s="68"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="68"/>
+      <c r="C34" s="68"/>
+      <c r="D34" s="87">
+        <f>+D29</f>
+        <v>36754.199999999997</v>
+      </c>
+      <c r="E34" s="68"/>
+      <c r="F34" s="68"/>
+      <c r="G34" s="68"/>
+      <c r="H34" s="68"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>